<commit_message>
rEEMPLAZO DLE DATO DLE NUMEERO DE REMITO EN PLANILLA ELENA
</commit_message>
<xml_diff>
--- a/ANDESMAR.xlsx
+++ b/ANDESMAR.xlsx
@@ -51,13 +51,13 @@
     <t>CÓRDOBA</t>
   </si>
   <si>
-    <t>01. Ventas Elena 1. 15-03-2022</t>
-  </si>
-  <si>
     <t>FULANO</t>
   </si>
   <si>
     <t>CODIGO POSTAL:</t>
+  </si>
+  <si>
+    <t>01. VTEL 1. 15-03-2022</t>
   </si>
 </sst>
 </file>
@@ -972,7 +972,7 @@
       <c r="C7" s="21"/>
       <c r="D7" s="8"/>
       <c r="E7" s="46" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F7" s="47"/>
       <c r="G7" s="47"/>
@@ -989,7 +989,7 @@
       <c r="C8" s="21"/>
       <c r="D8" s="10"/>
       <c r="E8" s="28" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F8" s="29"/>
       <c r="G8" s="29"/>
@@ -1069,7 +1069,7 @@
     <row r="13" spans="1:11" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="9"/>
       <c r="B13" s="44" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C13" s="45"/>
       <c r="D13" s="12"/>

</xml_diff>